<commit_message>
Adjust data validation helper text
</commit_message>
<xml_diff>
--- a/files/template-esp.xlsx
+++ b/files/template-esp.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jryan\Documents\R\projects\dirt-data-reports\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F122978C-BCDB-4F22-B042-79BD1A356663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFFE4023-A247-492F-8593-87CF3332D2F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-96" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="3" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="900" uniqueCount="451">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="452">
   <si>
     <t>year</t>
   </si>
@@ -1770,32 +1770,6 @@
   </si>
   <si>
     <t>Customize how the measurements appear in the Project Results section of the reports by editing the following columns:</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">• </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">measurement_group: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Defines how measurements are grouped into sections.</t>
-    </r>
   </si>
   <si>
     <r>
@@ -2022,7 +1996,124 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">    • Texture must be included in all datasets. The texture triangle used in the reports uses the USDA NRCS textural classification.</t>
+    <r>
+      <t xml:space="preserve">    • </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>texture</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> must be included in all datasets. The texture triangle used in the reports uses the USDA NRCS textural classification.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">    • </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>sand_percent</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>silt_percent</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>clay_percent</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> must be between 0 and 100.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">• </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">measurement_group: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Defines how measurements are grouped into sections. Allowable values are "Mediciones físicas", "Mediciones biológicas", "Mediciones químicas", "Macronutrientes esenciales para plantas", and "Micronutriente es esenciales para plantas".</t>
+    </r>
   </si>
   <si>
     <r>
@@ -2068,7 +2159,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> must be provided in decimal form.  Latitude must be between -90 and 90. Longitude must be between -180 and 180. Providing these coordinates is optional - if not included, no map will appear in the report.</t>
+      <t xml:space="preserve"> must be provided in decimal form. Latitude must be between -90 and 90. Longitude must be between -180 and 180. Providing these coordinates is optional. If they are not included, a map will not appear in the report.</t>
     </r>
   </si>
 </sst>
@@ -2454,10 +2545,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACB11E12-380E-4843-8FFB-3EEB7461C150}">
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="192" style="2" customWidth="1"/>
+    <col min="1" max="1" width="201" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
@@ -2477,12 +2568,12 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
@@ -2505,7 +2596,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>431</v>
       </c>
@@ -2545,9 +2636,9 @@
         <v>437</v>
       </c>
     </row>
-    <row r="21" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
@@ -2557,52 +2648,57 @@
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
         <v>449</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
-        <v>439</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
         <v>441</v>
       </c>
     </row>
-    <row r="28" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
+    <row r="29" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A29" s="1" t="s">
         <v>425</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A29" s="2" t="s">
-        <v>442</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>444</v>
+        <v>450</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>448</v>
+        <v>443</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>445</v>
+        <v>447</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
+        <v>444</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Use `soils::classify_texture()` (#64, #113)
Remove texture as required in template instructions
</commit_message>
<xml_diff>
--- a/files/template-esp.xlsx
+++ b/files/template-esp.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jryan\Documents\R\projects\dirt-data-reports\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFFE4023-A247-492F-8593-87CF3332D2F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{502451CE-2432-4D81-9DB0-9C70F5135F56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="3" r:id="rId1"/>
@@ -1997,6 +1997,32 @@
   </si>
   <si>
     <r>
+      <t xml:space="preserve">• </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">measurement_group: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Defines how measurements are grouped into sections. Allowable values are "Mediciones físicas", "Mediciones biológicas", "Mediciones químicas", "Macronutrientes esenciales para plantas", and "Micronutriente es esenciales para plantas".</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t xml:space="preserve">    • </t>
     </r>
     <r>
@@ -2008,7 +2034,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>texture</t>
+      <t>latitude</t>
     </r>
     <r>
       <rPr>
@@ -2018,7 +2044,96 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> must be included in all datasets. The texture triangle used in the reports uses the USDA NRCS textural classification.</t>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>longitude</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> must be provided in decimal form. Latitude must be between -90 and 90. Longitude must be between -180 and 180. Providing these coordinates is optional. If they are not included, a map will not appear in the report.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">    • texture may be left blank. If at least two of </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>sand_percent</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>silt_percent</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>clay_percent</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> are provided, texture will be classified according to the USDA NRCS.</t>
     </r>
   </si>
   <si>
@@ -2086,80 +2201,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> must be between 0 and 100.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">• </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">measurement_group: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Defines how measurements are grouped into sections. Allowable values are "Mediciones físicas", "Mediciones biológicas", "Mediciones químicas", "Macronutrientes esenciales para plantas", and "Micronutriente es esenciales para plantas".</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">    • </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>latitude</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> and </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>longitude</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> must be provided in decimal form. Latitude must be between -90 and 90. Longitude must be between -180 and 180. Providing these coordinates is optional. If they are not included, a map will not appear in the report.</t>
+      <t xml:space="preserve"> must be between 0 and 100 and sum to 100 (+/- 1). For each sample, at least two texture fractions must be provided (the third will be calculated as 100 minus the other two).</t>
     </r>
   </si>
 </sst>
@@ -2234,7 +2276,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2249,6 +2291,7 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2638,7 +2681,7 @@
     </row>
     <row r="21" spans="1:1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
@@ -2648,12 +2691,12 @@
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
     </row>
     <row r="24" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
@@ -2683,7 +2726,7 @@
     </row>
     <row r="31" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
@@ -2752,7 +2795,7 @@
       <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="6" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="4" t="s">
@@ -15062,7 +15105,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" deleteColumns="0" deleteRows="0"/>
+  <sheetProtection deleteColumns="0" deleteRows="0"/>
   <protectedRanges>
     <protectedRange sqref="K1:AW1048576" name="Measurements"/>
   </protectedRanges>
@@ -15540,7 +15583,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>

<commit_message>
Update helper text to remove texture as required
</commit_message>
<xml_diff>
--- a/files/template-esp.xlsx
+++ b/files/template-esp.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jryan\Documents\R\projects\dirt-data-reports\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{502451CE-2432-4D81-9DB0-9C70F5135F56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C049DDDC-697B-43FC-BD8B-67DB7870C056}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="3" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="452">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="900" uniqueCount="451">
   <si>
     <t>year</t>
   </si>
@@ -1903,78 +1903,6 @@
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>You need results from at least one soil sample for at least one soil health measurement, in addition to texture.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">• </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Texture is a required measurement and must be included in both the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> tab and the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dictionary</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> tab.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">• </t>
-    </r>
-    <r>
-      <rPr>
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
@@ -2066,74 +1994,6 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> must be provided in decimal form. Latitude must be between -90 and 90. Longitude must be between -180 and 180. Providing these coordinates is optional. If they are not included, a map will not appear in the report.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">    • texture may be left blank. If at least two of </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>sand_percent</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>silt_percent</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, and </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>clay_percent</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> are provided, texture will be classified according to the USDA NRCS.</t>
     </r>
   </si>
   <si>
@@ -2202,6 +2062,131 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> must be between 0 and 100 and sum to 100 (+/- 1). For each sample, at least two texture fractions must be provided (the third will be calculated as 100 minus the other two).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">    • </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>texture</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> may be left blank. If at least two of </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>sand_percent</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>silt_percent</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>clay_percent</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> are provided, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>texture</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> will be classified according to the USDA NRCS.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">• </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>You need results from at least one soil sample for at least one soil health measurement.</t>
     </r>
   </si>
 </sst>
@@ -2276,7 +2261,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2291,7 +2276,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2588,7 +2572,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACB11E12-380E-4843-8FFB-3EEB7461C150}">
-  <dimension ref="A1:A34"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="201" style="2" customWidth="1"/>
@@ -2611,141 +2595,137 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>445</v>
+        <v>450</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
         <v>430</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
+    <row r="10" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
         <v>423</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>431</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
         <v>432</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="3" t="s">
+    <row r="13" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
         <v>433</v>
       </c>
     </row>
-    <row r="16" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
+    <row r="15" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
         <v>424</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>434</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>449</v>
+        <v>438</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>451</v>
+        <v>439</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A27" s="2" t="s">
         <v>441</v>
       </c>
     </row>
-    <row r="29" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="1" t="s">
+    <row r="28" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="s">
         <v>425</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>448</v>
+        <v>443</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A34" s="2" t="s">
         <v>444</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2795,7 +2775,7 @@
       <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="4" t="s">

</xml_diff>

<commit_message>
Formatting tweaks to instructions
</commit_message>
<xml_diff>
--- a/files/template-esp.xlsx
+++ b/files/template-esp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jryan\Documents\R\projects\dirt-data-reports\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DB118C3-70E8-4F17-A287-7F1B9357A606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB60E879-61EB-4E29-9246-ECF379CEB55A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="5" r:id="rId1"/>
@@ -2222,30 +2222,6 @@
     <t>• Add columns for any additional measurements you wish to include.</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Important: Measurement column names in the Data tab must match exactly match the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <i/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>column_name</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> values in the Data Dictionary tab. Update the Data Dictionary tab after adding or removing measurements.</t>
-    </r>
-  </si>
-  <si>
     <t>Use the Data Dictionary to control how measurements appear in the Project Results section of the report.</t>
   </si>
   <si>
@@ -2457,12 +2433,42 @@
       <t>. Clean your data of common character values (e.g., ND, &lt;1) before uploading.</t>
     </r>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Important: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Measurement column names in the Data tab must match exactly match the </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>column_name</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> values in the Data Dictionary tab. Update the Data Dictionary tab after adding or removing measurements.</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -2488,13 +2494,6 @@
     <font>
       <b/>
       <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -2540,13 +2539,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <i/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -2591,22 +2583,22 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="2"/>
     </xf>
   </cellXfs>
@@ -2953,7 +2945,7 @@
     </row>
     <row r="9" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
@@ -3093,7 +3085,7 @@
     </row>
     <row r="41" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="9" t="s">
-        <v>457</v>
+        <v>466</v>
       </c>
     </row>
     <row r="43" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
@@ -3103,42 +3095,42 @@
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" s="6" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" s="10" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" s="11" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" s="11" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" s="6" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" s="6" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" s="6" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updates to template instructions
</commit_message>
<xml_diff>
--- a/files/template-esp.xlsx
+++ b/files/template-esp.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jryan\Documents\R\projects\dirt-data-reports\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB60E879-61EB-4E29-9246-ECF379CEB55A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9DD95FF-8D6D-4591-A0AC-F5FCA29C4C5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Instructions" sheetId="5" r:id="rId1"/>
+    <sheet name="Instructions" sheetId="7" r:id="rId1"/>
     <sheet name="Data" sheetId="1" r:id="rId2"/>
     <sheet name="Data Dictionary" sheetId="2" r:id="rId3"/>
   </sheets>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="467">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="918" uniqueCount="469">
   <si>
     <t>year</t>
   </si>
@@ -1753,63 +1753,6 @@
     <t>Review the example structure and format your project data to match.</t>
   </si>
   <si>
-    <r>
-      <t>Metadata</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> (columns A–I: </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>year</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> through </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>longitude</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>):</t>
-    </r>
-  </si>
-  <si>
     <t>• Do not delete metadata columns.</t>
   </si>
   <si>
@@ -2001,63 +1944,6 @@
         <family val="2"/>
       </rPr>
       <t>: -180 to 180.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Measurement results</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> (columns J–AO: </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>texture</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> through </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>na_mg_kg</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>):</t>
     </r>
   </si>
   <si>
@@ -2225,28 +2111,6 @@
     <t>Use the Data Dictionary to control how measurements appear in the Project Results section of the report.</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">• </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>measurement_group</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>: Defines how measurements are grouped into report sections.</t>
-    </r>
-  </si>
-  <si>
     <t>◦ Only the following values are currently supported. Custom groups are not allowed and will fail validation.</t>
   </si>
   <si>
@@ -2291,28 +2155,6 @@
         <family val="2"/>
       </rPr>
       <t>: Mediciones físicas, Mediciones biológicas, Mediciones químicas, Macronutrientes esenciales para plantas, Micronutrientes esenciales para plantas</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">• </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>column_name</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>: Links the Data tab to the Data Dictionary tab. Each measurement column header in the Data tab must have a matching entry here.</t>
     </r>
   </si>
   <si>
@@ -2463,6 +2305,230 @@
       <t xml:space="preserve"> values in the Data Dictionary tab. Update the Data Dictionary tab after adding or removing measurements.</t>
     </r>
   </si>
+  <si>
+    <r>
+      <t>Metadata</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (columns A–I: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>year</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> through </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>longitude</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>):</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Measurement results</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (columns J–AO: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>texture</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> through </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>na_mg_kg</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>):</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">• </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>measurement_group</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>: Defines how the soil measurements are grouped. Groups appear in the report in the order listed in the data dictionary.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">• </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>column_name</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>: Links the Data tab to the Data Dictionary tab. Must exactly match the column names of the soil measurements in your data. 
+   Within each measurement group, measurements appear in the order listed in the data dictionary.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">• All measurement columns </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>except texture</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> must be numeric. Non-numeric values (e.g., ND, &lt;1) will be coerced to NA and may be omitted from summaries, tables, and plots. Clean or recode censored values before uploading.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">• </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>abbr</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> + </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>unit</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>: Combination of abbreviation and unit be unique for each measurement.</t>
+    </r>
+  </si>
 </sst>
 </file>
 
@@ -2472,6 +2538,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2517,22 +2590,14 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="12"/>
+      <i/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -2566,8 +2631,9 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="12">
@@ -2575,36 +2641,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="2"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{FE0BADA4-05D1-421C-967F-EE13CEF2E860}"/>
+    <cellStyle name="Normal 2 2" xfId="2" xr:uid="{7FB901AB-5CAF-43B9-B7B0-EB2877FC51F8}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2897,8 +2964,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0AD959F-2200-4584-B3C1-B4547058E3E9}">
-  <dimension ref="A1:A51"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EEC8161-8920-4FDF-86E6-C9DCD5CCCF40}">
+  <dimension ref="A1:A53"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="176.33203125" style="4" customWidth="1"/>
@@ -2945,7 +3012,7 @@
     </row>
     <row r="9" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
@@ -2983,154 +3050,164 @@
         <v>436</v>
       </c>
     </row>
-    <row r="20" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="3" t="s">
-        <v>437</v>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" s="8" t="s">
+        <v>463</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" s="7" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" s="8" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" s="7" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" s="7" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" s="7" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="3" t="s">
-        <v>449</v>
+        <v>447</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A33" s="8" t="s">
+        <v>464</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A34" s="6" t="s">
-        <v>450</v>
+      <c r="A34" t="s">
+        <v>467</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A36" s="7" t="s">
-        <v>452</v>
+      <c r="A36" s="6" t="s">
+        <v>449</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" s="7" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" s="7" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A39" s="6" t="s">
-        <v>455</v>
+      <c r="A39" s="7" t="s">
+        <v>452</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" s="6" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="9" t="s">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A43" s="3" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A41" s="6" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="9" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A44" s="3" t="s">
         <v>424</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A44" s="6" t="s">
-        <v>457</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A46" s="10" t="s">
-        <v>459</v>
+      <c r="A46" s="6" t="s">
+        <v>465</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A47" s="11" t="s">
-        <v>460</v>
+      <c r="A47" s="10" t="s">
+        <v>456</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" s="11" t="s">
-        <v>461</v>
+        <v>457</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A49" s="6" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49" s="11" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A50" s="6" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" s="6" t="s">
-        <v>464</v>
+        <v>459</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A52" s="6" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A53" s="6" t="s">
+        <v>468</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Use "convert" instead of "coerce"
</commit_message>
<xml_diff>
--- a/files/template-esp.xlsx
+++ b/files/template-esp.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jryan\Documents\R\projects\dirt-data-reports\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9DD95FF-8D6D-4591-A0AC-F5FCA29C4C5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37643283-F070-4845-98D1-CB96E621DC86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="7" r:id="rId1"/>
@@ -2203,6 +2203,260 @@
   </si>
   <si>
     <r>
+      <t xml:space="preserve">Important: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Measurement column names in the Data tab must match exactly match the </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>column_name</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> values in the Data Dictionary tab. Update the Data Dictionary tab after adding or removing measurements.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Metadata</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (columns A–I: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>year</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> through </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>longitude</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>):</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Measurement results</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (columns J–AO: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>texture</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> through </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>na_mg_kg</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>):</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">• </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>measurement_group</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>: Defines how the soil measurements are grouped. Groups appear in the report in the order listed in the data dictionary.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">• </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>column_name</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>: Links the Data tab to the Data Dictionary tab. Must exactly match the column names of the soil measurements in your data. 
+   Within each measurement group, measurements appear in the order listed in the data dictionary.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">• All measurement columns </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>except texture</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> must be numeric. Non-numeric values (e.g., ND, &lt;1) will be coerced to NA and may be omitted from summaries, tables, and plots. Clean or recode censored values before uploading.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">• </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>abbr</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> + </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>unit</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>: Combination of abbreviation and unit be unique for each measurement.</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t xml:space="preserve">◦ Measurement results (e.g., </t>
     </r>
     <r>
@@ -2264,7 +2518,7 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>Non-numeric values will be coerced to NA</t>
+      <t>Non-numeric values will be converted to NA</t>
     </r>
     <r>
       <rPr>
@@ -2275,266 +2529,12 @@
       <t>. Clean your data of common character values (e.g., ND, &lt;1) before uploading.</t>
     </r>
   </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Important: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Measurement column names in the Data tab must match exactly match the </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>column_name</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> values in the Data Dictionary tab. Update the Data Dictionary tab after adding or removing measurements.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Metadata</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> (columns A–I: </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>year</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> through </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>longitude</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>):</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Measurement results</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> (columns J–AO: </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>texture</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> through </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>na_mg_kg</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>):</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">• </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>measurement_group</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>: Defines how the soil measurements are grouped. Groups appear in the report in the order listed in the data dictionary.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">• </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>column_name</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>: Links the Data tab to the Data Dictionary tab. Must exactly match the column names of the soil measurements in your data. 
-   Within each measurement group, measurements appear in the order listed in the data dictionary.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">• All measurement columns </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>except texture</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> must be numeric. Non-numeric values (e.g., ND, &lt;1) will be coerced to NA and may be omitted from summaries, tables, and plots. Clean or recode censored values before uploading.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">• </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>abbr</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> + </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>unit</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>: Combination of abbreviation and unit be unique for each measurement.</t>
-    </r>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -2591,13 +2591,6 @@
     </font>
     <font>
       <i/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -3012,7 +3005,7 @@
     </row>
     <row r="9" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
-        <v>461</v>
+        <v>468</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
@@ -3052,7 +3045,7 @@
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
@@ -3112,12 +3105,12 @@
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="8" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
@@ -3157,7 +3150,7 @@
     </row>
     <row r="42" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="44" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
@@ -3172,7 +3165,7 @@
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
@@ -3192,7 +3185,7 @@
     </row>
     <row r="50" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A50" s="6" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
@@ -3207,7 +3200,7 @@
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" s="6" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update templates and helper modals
</commit_message>
<xml_diff>
--- a/files/template-esp.xlsx
+++ b/files/template-esp.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jryan\Documents\R\projects\dirt-data-reports\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jryan\Documents\R\projects\soils\inst\templates\spanish\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37643283-F070-4845-98D1-CB96E621DC86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5DADA1B-89CD-443E-981F-6C364C46A238}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="918" uniqueCount="469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="915" uniqueCount="466">
   <si>
     <t>year</t>
   </si>
@@ -2111,53 +2111,6 @@
     <t>Use the Data Dictionary to control how measurements appear in the Project Results section of the report.</t>
   </si>
   <si>
-    <t>◦ Only the following values are currently supported. Custom groups are not allowed and will fail validation.</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">▪ </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>English</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>: Physical, Biological, Chemical, Plant Essential Macro Nutrients, Plant Essential Micro Nutrients</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">▪ </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Spanish</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>: Mediciones físicas, Mediciones biológicas, Mediciones químicas, Macronutrientes esenciales para plantas, Micronutrientes esenciales para plantas</t>
-    </r>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">• </t>
     </r>
@@ -2629,7 +2582,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -2653,12 +2606,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1" indent="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2958,7 +2905,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EEC8161-8920-4FDF-86E6-C9DCD5CCCF40}">
-  <dimension ref="A1:A53"/>
+  <dimension ref="A1:A50"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="176.33203125" style="4" customWidth="1"/>
@@ -3005,7 +2952,7 @@
     </row>
     <row r="9" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
@@ -3045,7 +2992,7 @@
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
@@ -3105,12 +3052,12 @@
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="8" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
@@ -3150,7 +3097,7 @@
     </row>
     <row r="42" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
     </row>
     <row r="44" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
@@ -3165,42 +3112,27 @@
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A47" s="6" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A48" s="6" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49" s="6" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A50" s="6" t="s">
         <v>464</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A47" s="10" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A48" s="11" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A49" s="11" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A50" s="6" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A51" s="6" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A52" s="6" t="s">
-        <v>460</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A53" s="6" t="s">
-        <v>467</v>
       </c>
     </row>
   </sheetData>

</xml_diff>